<commit_message>
feat: add JWT revocation and session security tests
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
+++ b/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
@@ -466,7 +466,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -647,7 +647,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -826,7 +826,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -1003,7 +1003,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -1180,7 +1180,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
@@ -1233,7 +1233,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
@@ -1265,7 +1265,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="pt-PT"/>
         </a:p>
@@ -3522,12 +3522,12 @@
       </c>
       <c r="F8" s="39" t="inlineStr">
         <is>
-          <t>Partially Compliant</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>JWT MAC, HS256 allowlist and exp validation exist; issuer/audience claims, key rotation and token denylist are pending.</t>
+          <t>JWTs now validate typ, algorithm, exp, issuer, audience and jti before authentication is accepted.</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -3562,12 +3562,12 @@
       </c>
       <c r="F9" s="39" t="inlineStr">
         <is>
-          <t>Partially Compliant</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>JWT MAC, HS256 allowlist and exp validation exist; issuer/audience claims, key rotation and token denylist are pending.</t>
+          <t>JWT audience is fixed to ghostreport-api and validated by JwtService tests.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>JWT MAC, HS256 allowlist and exp validation exist; issuer/audience claims, key rotation and token denylist are pending.</t>
+          <t>Issuer and audience are present and validated. Key rotation and separate signing keys for multiple audiences are outside the current local-JWT design.</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/test/java/com/ghostreport/security/JwtServiceSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/service/JwtService.java</t>
         </is>
       </c>
     </row>
@@ -11197,7 +11197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11303,6 +11303,20 @@
       <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Project.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Phase 7 update - JWT/session management</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Added logout-driven JWT revocation, jti, issuer and audience validation, frontend logout calls, and tests for revoked-token reuse. V7/V9 remain partially compliant overall because refresh-token rotation, concurrent-session management, distributed revocation and key rotation are not implemented.</t>
         </is>
       </c>
     </row>
@@ -16391,12 +16405,12 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>BCrypt, inactive-user checks and login rate limiting exist; MFA, password reset, password history and stronger lockout remain future work.</t>
+          <t>Rate limiting, invalid-login audit and logout audit are implemented and tested. MFA/password recovery controls remain documented gaps.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/AuthService.java; ghostreport/src/test/java/com/ghostreport/security/LoginRateLimitSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/test/java/com/ghostreport/security/LoginRateLimitSecurityTest.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -17027,7 +17041,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Login abuse is rate limited and covered by security tests.</t>
+          <t>Login brute-force protection is implemented with rate limiting and security alerts; tests cover repeated failures and 429 response.</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
@@ -18676,12 +18690,12 @@
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>JWT stateless session validates signature, expiry and role; logout revocation/denylist and refresh-token rotation are pending.</t>
+          <t>Self-contained JWTs are dynamically generated and now include exp, iss, aud and jti. Access-token refresh rotation is not implemented.</t>
         </is>
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/test/java/com/ghostreport/security/JwtServiceSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/test/java/com/ghostreport/security/JwtServiceSecurityTest.java</t>
         </is>
       </c>
     </row>
@@ -18756,12 +18770,12 @@
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>JWT stateless session validates signature, expiry and role; logout revocation/denylist and refresh-token rotation are pending.</t>
+          <t>A new JWT is issued on login and explicit logout revokes the current token. The application does not automatically terminate all previously issued tokens on re-authentication.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/test/java/com/ghostreport/security/JwtServiceSecurityTest.java</t>
+          <t>ghostreport/src/main/java/com/ghostreport/controller/AuthController.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -18907,17 +18921,17 @@
       </c>
       <c r="F15" s="41" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Server-side token revocation/logout is not implemented yet.</t>
+          <t>Explicit logout revokes the JWT jti and tests prove the same Bearer token is rejected after logout.</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>docs/ASVS_EVIDENCE.md</t>
+          <t>ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/main/java/com/ghostreport/controller/AuthController.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -19027,17 +19041,17 @@
       </c>
       <c r="F18" s="41" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partially Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Server-side token revocation/logout is not implemented yet.</t>
+          <t>Authenticated role dashboards expose logout actions and frontend logout calls POST /auth/logout before clearing browser storage. Coverage is limited to current dashboards.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>docs/ASVS_EVIDENCE.md</t>
+          <t>ghostreport/src/main/resources/static/js/admin.js; ghostreport/src/main/resources/static/js/analyst.js; ghostreport/src/main/resources/static/js/auditor.js</t>
         </is>
       </c>
     </row>
@@ -19170,12 +19184,12 @@
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>JWT stateless session validates signature, expiry and role; logout revocation/denylist and refresh-token rotation are pending.</t>
+          <t>Users can terminate the current token through logout. Viewing and terminating all concurrent sessions is not implemented.</t>
         </is>
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/JwtService.java; ghostreport/src/test/java/com/ghostreport/security/JwtServiceSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/controller/AuthController.java</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: harden authentication controls
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
+++ b/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
@@ -11197,7 +11197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11317,6 +11317,20 @@
       <c r="A20" t="inlineStr">
         <is>
           <t>Added logout-driven JWT revocation, jti, issuer and audience validation, frontend logout calls, and tests for revoked-token reuse. V7/V9 remain partially compliant overall because refresh-token rotation, concurrent-session management, distributed revocation and key rotation are not implemented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Phase 8 update - authentication hardening</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Login rate limiting is now scoped by normalized username and client IP, reducing account-specific brute-force risk without locking out unrelated users behind the same address. MFA and password recovery remain residual gaps.</t>
         </is>
       </c>
     </row>
@@ -17041,12 +17055,12 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Login brute-force protection is implemented with rate limiting and security alerts; tests cover repeated failures and 429 response.</t>
+          <t>Login brute-force protection is implemented with username/IP-scoped rate limiting and security alerts; tests cover repeated failures, 429 response and isolation between users sharing the same IP.</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/RateLimiterService.java; ghostreport/src/test/java/com/ghostreport/security/LoginRateLimitSecurityTest.java</t>
+          <t>ghostreport/src/main/java/com/ghostreport/controller/AuthController.java; ghostreport/src/main/java/com/ghostreport/service/RateLimiterService.java; ghostreport/src/test/java/com/ghostreport/security/LoginRateLimitSecurityTest.java</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: improve coverage for critical security flows
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
+++ b/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
@@ -9831,12 +9831,12 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Audit logs, security alerts and generic errors are implemented; centralized SIEM/tamper-resistant logging and incident runbooks are pending.</t>
+          <t>Audit/security events are recorded and exposed through ADMIN-only DTO endpoints; tests cover login/logout/invalid JWT and admin evidence retrieval. Centralized SIEM, tamper resistance and full incident runbooks are not implemented.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/AuditLogService.java; ghostreport/src/main/java/com/ghostreport/service/SecurityMonitoringService.java; ghostreport/src/test/java/com/ghostreport/security/ErrorHandlingSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/controller/AdminController.java; ghostreport/src/test/java/com/ghostreport/security/AdminUserManagementSecurityTest.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -9889,12 +9889,12 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Audit logs, security alerts and generic errors are implemented; centralized SIEM/tamper-resistant logging and incident runbooks are pending.</t>
+          <t>Audit/security events are recorded and exposed through ADMIN-only DTO endpoints; tests cover login/logout/invalid JWT and admin evidence retrieval. Centralized SIEM, tamper resistance and full incident runbooks are not implemented.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/AuditLogService.java; ghostreport/src/main/java/com/ghostreport/service/SecurityMonitoringService.java; ghostreport/src/test/java/com/ghostreport/security/ErrorHandlingSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/controller/AdminController.java; ghostreport/src/test/java/com/ghostreport/security/AdminUserManagementSecurityTest.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -9929,12 +9929,12 @@
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>Audit logs, security alerts and generic errors are implemented; centralized SIEM/tamper-resistant logging and incident runbooks are pending.</t>
+          <t>Audit/security events are recorded and exposed through ADMIN-only DTO endpoints; tests cover login/logout/invalid JWT and admin evidence retrieval. Centralized SIEM, tamper resistance and full incident runbooks are not implemented.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>ghostreport/src/main/java/com/ghostreport/service/AuditLogService.java; ghostreport/src/main/java/com/ghostreport/service/SecurityMonitoringService.java; ghostreport/src/test/java/com/ghostreport/security/ErrorHandlingSecurityTest.java</t>
+          <t>docs/ASVS_EVIDENCE.md; ghostreport/src/main/java/com/ghostreport/controller/AdminController.java; ghostreport/src/test/java/com/ghostreport/security/AdminUserManagementSecurityTest.java; ghostreport/src/test/java/com/ghostreport/security/RuntimeSecurityEventLoggingTest.java</t>
         </is>
       </c>
     </row>
@@ -11197,7 +11197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11331,6 +11331,20 @@
       <c r="A23" t="inlineStr">
         <is>
           <t>Login rate limiting is now scoped by normalized username and client IP, reducing account-specific brute-force risk without locking out unrelated users behind the same address. MFA and password recovery remain residual gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Phase 9 update - critical security-flow coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Added MockMvc coverage for ADMIN retrieval of audit logs and security alerts as DTOs, strengthening V16 evidence and admin controller coverage. Overall V16 remains partial due missing tamper-resistant logging/SIEM.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: archive post-remediation dependency scan
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
+++ b/Deliverables/Phase 2/ASVS_5.0_Tracker_Phase 2_Sprint 2.xlsx
@@ -8835,12 +8835,12 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -8875,12 +8875,12 @@
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -8915,12 +8915,12 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -8955,12 +8955,12 @@
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -8995,12 +8995,12 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9053,12 +9053,12 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9093,12 +9093,12 @@
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9133,12 +9133,12 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9173,12 +9173,12 @@
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9213,12 +9213,12 @@
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9271,12 +9271,12 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9311,12 +9311,12 @@
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9351,12 +9351,12 @@
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9391,12 +9391,12 @@
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9431,12 +9431,12 @@
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9471,12 +9471,12 @@
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9511,12 +9511,12 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9569,12 +9569,12 @@
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9609,12 +9609,12 @@
       </c>
       <c r="G24" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H24" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9649,12 +9649,12 @@
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H25" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -9689,12 +9689,12 @@
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>SAST, SCA, SBOM, DAST, Gitleaks and testing evidence exist; Dependency-Check and SpotBugs findings remain open.</t>
+          <t>Post-remediation Dependency-Check evidence exists and major Spring Boot/Tomcat/PostgreSQL/Log4j findings were removed; angus-activation and hibernate-validator remain residual-risk triage items.</t>
         </is>
       </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
-          <t>.github/workflows; Deliverables/Phase 2/Evidence/sast; Deliverables/Phase 2/Evidence/sca</t>
+          <t>docs/SCA_TRIAGE.md; Deliverables/Phase 2/Evidence/sca/dependency-check-post-remediation; docs/ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -11197,7 +11197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11345,6 +11345,20 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>Added MockMvc coverage for ADMIN retrieval of audit logs and security alerts as DTOs, strengthening V16 evidence and admin controller coverage. Overall V16 remains partial due missing tamper-resistant logging/SIEM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Final validation update - SCA post-remediation evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Local Dependency-Check completed successfully after dependency updates. Evidence archived under sca/dependency-check-post-remediation. Remaining findings: angus-activation CVE-2025-7962 and hibernate-validator CVE-2025-15104 under manual residual-risk triage.</t>
         </is>
       </c>
     </row>

</xml_diff>